<commit_message>
refactor: centralize the complete scoring rubric
</commit_message>
<xml_diff>
--- a/audit_risk_register.xlsx
+++ b/audit_risk_register.xlsx
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -875,7 +875,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>发生可能性（1-5）</t>
+          <t>发生可能性</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>COSO ERM 2017 风险偏好校准</t>
+          <t>COSO ERM 2017</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>内审发现/监管检查通报</t>
+          <t>内审发现/监管通报</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>ACFE：组织年均约 5% 收入流失于舞弊</t>
+          <t>ACFE：年均约 5% 营收流失于舞弊</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>已多次发生或正在发生，相关控制基本失效</t>
+          <t>已多次发生或正在发生，控制基本失效</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -974,7 +974,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>经济损失 —— 国资委资产损失分级 + 国务院令第 493 号</t>
+          <t>经济损失（国资委资产损失分级 + 493 号令）</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>&lt;100 万元：未达“一般资产损失”标准，企业内部可消化</t>
+          <t>&lt;100 万元：未达“一般资产损失”</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>100~500 万元：构成“一般资产损失”</t>
+          <t>100~500 万元：一般资产损失</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>国资委办法：&lt;500 万为一般</t>
+          <t>国资委办法</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>500~5000 万元：构成“较大资产损失”；493 号令“较大事故”直接损失落于本档</t>
+          <t>500~5000 万元：较大资产损失；较大事故损失区间</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>国资委办法；国务院令第 493 号</t>
+          <t>国资委办法；493 号令</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>5000 万~1 亿元：构成“重大资产损失”；493 号令“重大事故”量级</t>
+          <t>5000 万~1 亿元：重大资产损失；重大事故量级</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>≥1 亿元：493 号令“特别重大事故”量级，危及企业生存</t>
+          <t>≥1 亿元：特别重大事故量级，危及企业生存</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1073,7 +1073,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>合规法律 —— 个保法/数安法/GDPR + 国资委不良后果三档</t>
+          <t>合规法律（个保法/数安法/GDPR + 不良后果三档）</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>内部制度瑕疵，责令整改即可，无外部后果</t>
+          <t>制度瑕疵，责令整改，无外部后果</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>监管关注/责令限期整改；罚款 &lt;100 万元</t>
+          <t>责令限期整改；罚款 &lt;100 万元</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>一般行政处罚，罚款 100~1000 万元；责任人被处分</t>
+          <t>一般行政处罚 100~1000 万元；责任人被处分</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>数安法第 45 条；网数条例第 56 条</t>
+          <t>数安法第 45 条</t>
         </is>
       </c>
     </row>
@@ -1145,12 +1145,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>情节严重：罚款 1000~5000 万或上年营业额 5%（GDPR 顶格 2000 万欧/4% 同档）</t>
+          <t>情节严重 1000~5000 万或营业额 5%（GDPR 顶格同档）</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>个保法第 66 条第二款；GDPR Art.83</t>
+          <t>个保法第 66 条第二款；GDPR</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>刑事责任移送、责令停业/吊销执照；影响社会与国家层面</t>
+          <t>刑事移送、停业/吊照；影响社会与国家层面</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>运营中断 —— 493 号令事故等级 + ISO 22301 RTO 分级</t>
+          <t>运营中断（493 号令事故等级 + ISO 22301 RTO）</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>局部岗位受阻，当日恢复（RTO&lt;8h），无人员伤害</t>
+          <t>局部受阻，当日恢复（RTO&lt;8h）</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>ISO 22301 恢复目标分级</t>
+          <t>ISO 22301</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>单部门中断，RTO 1~3 天；轻微伤害事件</t>
+          <t>单部门中断，RTO 1~3 天</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>跨部门/跨区域中断，RTO 3~30 天；或 493 号令“一般事故”</t>
+          <t>跨部门中断，RTO 3~30 天；或“一般事故”</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>核心业务瘫痪 1~6 个月；或“较大/重大事故”量级</t>
+          <t>核心业务瘫痪 1~6 个月；或较大/重大事故量级</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>集团级瘫痪超 6 个月；或“特别重大事故”（≥30 人死亡或≥1 亿元）</t>
+          <t>集团级瘫痪超 6 个月；或特别重大事故</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -1271,7 +1271,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>声誉舆情 —— 国资委不良后果三档 × 传播层级</t>
+          <t>声誉舆情（国资委不良后果三档 × 传播层级）</t>
         </is>
       </c>
     </row>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>个别投诉、本地媒体负面报道，影响限于涉事企业</t>
+          <t>个别投诉、本地媒体报道，影响限于涉事企业</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>国资委：一般不良后果</t>
+          <t>一般不良后果</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>行业内流传、省级媒体或行业监管通报</t>
+          <t>行业内流传、省级媒体/监管通报</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>国资委：较大不良后果</t>
+          <t>较大不良后果</t>
         </is>
       </c>
     </row>
@@ -1343,12 +1343,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>全国性媒体报道、上级通报批评，资本市场负面反应</t>
+          <t>全国性报道、上级通报批评、资本市场负面反应</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>国资委：较大~重大不良后果</t>
+          <t>较大~重大不良后果</t>
         </is>
       </c>
     </row>
@@ -1358,19 +1358,19 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>国家级媒体/监管部门点名、社会舆论事件、引发行业整顿</t>
+          <t>国家级点名、社会舆论事件、行业整顿</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>国资委：重大不良后果</t>
+          <t>重大不良后果</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>舞弊风险 —— ACFE 2024 基准 + 监察机关职务犯罪管辖</t>
+          <t>舞弊风险（ACFE 2024 基准 + 职务犯罪管辖）</t>
         </is>
       </c>
     </row>
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>无舞弊诱因，职责分离健全且经穿行测试，无历史案例</t>
+          <t>无诱因，职责分离健全经测试，无案例</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>COSO 控制环境；ISO 37001</t>
+          <t>COSO；ISO 37001</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>ACFE 2024：中位损失 $14.5 万</t>
+          <t>ACFE：中位 $14.5 万</t>
         </is>
       </c>
     </row>
@@ -1427,12 +1427,12 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>诱因集中（权限集中/监督薄弱）；潜在损失 100~500 万元</t>
+          <t>诱因集中；潜在损失 100~500 万元</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>ACFE 2024：75 分位 $75 万</t>
+          <t>ACFE：75 分位 $75 万</t>
         </is>
       </c>
     </row>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>诱因高危或有历史案例；潜在损失 500~5000 万元；涉嫌职务违法</t>
+          <t>诱因高危或有案例；潜在损失 500~5000 万元</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>国资委较大~重大资产损失档</t>
+          <t>国资委较大~重大档</t>
         </is>
       </c>
     </row>
@@ -1462,68 +1462,365 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>ACFE：年均 5% 收入流失于舞弊</t>
+          <t>ACFE：年均 5% 营收</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>战略影响（COSO ERM + 央企指引战略风险）</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>分值</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>锚点</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>权威依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>对战略目标无偏离影响</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>COSO ERM 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>影响单项年度 KPI，可内部消化</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>COSO ERM 战略类</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>影响年度重点战略举措推进</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>央企指引战略风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>影响三年规划目标或主营业务布局</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>COSO：战略与绩效</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>颠覆战略目标/主营业务模式重构</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>央企指引：战略风险重大</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>数据安全（数安法分级 + ISO 27001 CIA）</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>分值</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>锚点</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>权威依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>不涉及敏感数据</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>ISO 27001</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>少量内部非敏数据受损，可恢复</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>网数条例第 57 条</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>一般个人信息或商业数据泄露（&lt;10 万条）</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>个保法第 66 条第一款</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>大量个人信息/重要数据泄露或出境违规</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>个保法顶格；数安法第 45 条</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>重要数据泄露危害国家安全/公共安全</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>数安法：重大违规</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>健康安全（ISO 45001 + 安全生产法 + 493 号令）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>分值</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>锚点</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>权威依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>无人员伤害可能</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>ISO 45001</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>轻微伤风险，职业健康隐患</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>ISO 45001</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>重伤风险；一般事故苗头（&lt;3 人死亡）</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>493 号令一般事故</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>死亡 3~30 人或重伤 10~100 人量级</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>493 号令较大/重大事故</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>群死群伤（≥30 人死亡）或特别重大事故</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>493 号令特别重大</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
           <t>权威来源</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>1. 国务院国资委《中央企业违规经营投资责任追究实施办法》（2025 年修订，2026-01-01 施行，替代 37 号令）</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>2. 国务院令第 493 号《生产安全事故报告和调查处理条例》</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>3. 《个人信息保护法》第 66 条、《数据安全法》第 45 条、《网络数据安全管理条例》</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>4. GDPR 第 83 条（2000 万欧元或全球营业额 4%）</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>5. ACFE《Occupational Fraud 2024: A Report to the Nations》</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>6. 《监察法》《刑法》职务犯罪管辖标准</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>7. ISO 31000 / ISO 37301 / ISO 37001 / ISO 22301</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>8. COSO ERM 2017、IIA《全球内部审计准则》（2024）</t>
         </is>

</xml_diff>